<commit_message>
Remove duplicate fw111 listing from gallery data
</commit_message>
<xml_diff>
--- a/s/lorelei-wood-etsy-image-rescue/downloads/Shopify_Copy_Sheet.xlsx
+++ b/s/lorelei-wood-etsy-image-rescue/downloads/Shopify_Copy_Sheet.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M42"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2656,86 +2656,15 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>fw111thset_batch_22</t>
+          <t>fw112thset_batch_03</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>XL soft and plush "Sherbert Peavock" vintage chenille bathrobe upcycled from hand tufted chenille bedspreads The colors in this bathrobe remind me of rainbow sherbet, so pretty and pastel. The</t>
+          <t>Medium heavy and plush "Peachy Triple Peacock" vintage chenille bathrobe upcycled from hand tufted 'double' chenille bedspread Heavy 'double' chenille; which has the background chenille created by the manufacturer,</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Vy o
-The colors in this bathrobe remind me of rainbow sherbet, so pretty and pastel. The
-peacock on the back is simply gorgeous, very thickly tufted; and so thick you cannot see
-the backing in between the lines of chenille. The peacock is surrounded by a peach
-trellis and purple roses on the trellis. I chose purple for the sleeves to pick up those rose
-colors.
-XL can fit up to a woman's size 24. with pockets; machine washable too.
-Chenille bedspreads were created and manufactured in the US during the 1930s to the
-1950s; much of it was hand tufted. The hand tufting process was often a series of knots
-tied in a pre-printed design onto cotton (muslin) fabric. These one-of-a-kind bedspreads
-varied by the tufter, as well as by materials used.
-The production of chenille stopped in the United States after about 1960, and much of it
-is being up cycled and given new life. Since the supply of vintage chenille is limited and
-finite, it has become more difficult to find! Although chenille is durable, it can suffer
-wear over time that may take the form of thinning lines of chenille, skipped spots where</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>vintage, chenille, bathrobe, robe, upcycled, bedspread, peacock, rose, cotton, hand tufted, plush</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>xl-soft-and-plush-sherbert-peavock-vintage-chenille-bathrobe-upcycled-from-hand</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>02_All_Listings_By_Set/fw111thset_batch_22/Cropped_Images</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>fw111thset_batch_22_xl-soft-and-plush-sherbert-peavock-vintage-chenille-bathrobe_img01_2026-05-27_164908.png</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>fw111thset_batch_22_xl-soft-and-plush-sherbert-peavock-vintage-chenille-bathrobe_img01_2026-05-27_164908.png | fw111thset_batch_22_xl-soft-and-plush-sherbert-peavock-vintage-chenille-bathrobe_img02_2026-05-27_164908.png | fw111thset_batch_22_xl-soft-and-plush-sherbert-peavock-vintage-chenille-bathrobe_img03_2026-05-27_164914.png | fw111thset_batch_22_xl-soft-and-plush-sherbert-peavock-vintage-chenille-bathrobe_img04_2026-05-27_164925.png | fw111thset_batch_22_xl-soft-and-plush-sherbert-peavock-vintage-chenille-bathrobe_img05_2026-05-27_164931.png | fw111thset_batch_22_xl-soft-and-plush-sherbert-peavock-vintage-chenille-bathrobe_img06_2026-05-27_164935.png | fw111thset_batch_22_xl-soft-and-plush-sherbert-peavock-vintage-chenille-bathrobe_img07_2026-05-27_164940.png | fw111thset_batch_22_xl-soft-and-plush-sherbert-peavock-vintage-chenille-bathrobe_img08_2026-05-27_164945.png | fw111thset_batch_22_xl-soft-and-plush-sherbert-peavock-vintage-chenille-bathrobe_img09_2026-05-27_164951.png</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>Screenshot 2026-05-27 at 4.49.08 PM.png: needs_review - Automatic crop passed layout checks. Possible Etsy overlay inside product photo. | Screenshot 2026-05-27 at 4.49.08 PM_1.png: needs_review - Automatic crop passed layout checks. Possible Etsy overlay inside product photo.</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>fw112thset_batch_03</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Medium heavy and plush "Peachy Triple Peacock" vintage chenille bathrobe upcycled from hand tufted 'double' chenille bedspread Heavy 'double' chenille; which has the background chenille created by the manufacturer,</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Heavy 'double' chenille; which has the background chenille created by the manufacturer,
 and the hand tufted design on top of the manufactured chenille tufting. Gorgeous
@@ -2753,59 +2682,59 @@
 wear over time that may take the form of thinning lines of chenille, skipped spots where</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>vintage, chenille, bathrobe, robe, upcycled, bedspread, peacock, flower, cotton, hand tufted, plush, heavy</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>medium-heavy-and-plush-peachy-triple-peacock-vintage-chenille-bathrobe-upcycled</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>02_All_Listings_By_Set/fw112thset_batch_03/Cropped_Images</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>fw112thset_batch_03_medium-heavy-and-plush-peachy-triple-peacock-vintage-chenill_img01_2026-05-27_164740.png</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>fw112thset_batch_03_medium-heavy-and-plush-peachy-triple-peacock-vintage-chenill_img01_2026-05-27_164740.png | fw112thset_batch_03_medium-heavy-and-plush-peachy-triple-peacock-vintage-chenill_img02_2026-05-27_164747.png | fw112thset_batch_03_medium-heavy-and-plush-peachy-triple-peacock-vintage-chenill_img03_2026-05-27_164752.png | fw112thset_batch_03_medium-heavy-and-plush-peachy-triple-peacock-vintage-chenill_img04_2026-05-27_164756.png | fw112thset_batch_03_medium-heavy-and-plush-peachy-triple-peacock-vintage-chenill_img05_2026-05-27_164801.png | fw112thset_batch_03_medium-heavy-and-plush-peachy-triple-peacock-vintage-chenill_img06_2026-05-27_164806.png | fw112thset_batch_03_medium-heavy-and-plush-peachy-triple-peacock-vintage-chenill_img07_2026-05-27_164811.png | fw112thset_batch_03_medium-heavy-and-plush-peachy-triple-peacock-vintage-chenill_img08_2026-05-27_164817.png | fw112thset_batch_03_medium-heavy-and-plush-peachy-triple-peacock-vintage-chenill_img09_2026-05-27_164822.png</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>Screenshot 2026-05-27 at 4.47.40 PM.png: needs_review - Automatic crop passed layout checks. Possible Etsy overlay inside product photo.</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr"/>
-      <c r="M34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>fw114thset_batch_04</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Small heavy "Dusty Rose Quadruple Peacock" chenille bathrobe upcycled from vintage hand tufted chenille bedspreads</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>This small can fit up to a woman's size 8, with pockets. Four (!) peacocks...large one in
 the back, another large one AND two more tiny ones in the front! The chenille used in
@@ -2820,59 +2749,59 @@
 garment.</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>vintage, chenille, bathrobe, robe, upcycled, bedspread, peacock, rose, hand tufted, heavy</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>small-heavy-dusty-rose-quadruple-peacock-chenille-bathrobe-upcycled-from-vintage</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>02_All_Listings_By_Set/fw114thset_batch_04/Cropped_Images</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>fw114thset_batch_04_small-heavy-dusty-rose-quadruple-peacock-chenille-bathrobe-u_img01_2026-05-27_195349.png</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>fw114thset_batch_04_small-heavy-dusty-rose-quadruple-peacock-chenille-bathrobe-u_img01_2026-05-27_195349.png | fw114thset_batch_04_small-heavy-dusty-rose-quadruple-peacock-chenille-bathrobe-u_img02_2026-05-27_195355.png | fw114thset_batch_04_small-heavy-dusty-rose-quadruple-peacock-chenille-bathrobe-u_img03_2026-05-27_195359.png | fw114thset_batch_04_small-heavy-dusty-rose-quadruple-peacock-chenille-bathrobe-u_img04_2026-05-27_195404.png | fw114thset_batch_04_small-heavy-dusty-rose-quadruple-peacock-chenille-bathrobe-u_img05_2026-05-27_195410.png | fw114thset_batch_04_small-heavy-dusty-rose-quadruple-peacock-chenille-bathrobe-u_img06_2026-05-27_195416.png | fw114thset_batch_04_small-heavy-dusty-rose-quadruple-peacock-chenille-bathrobe-u_img07_2026-05-27_195421.png | fw114thset_batch_04_small-heavy-dusty-rose-quadruple-peacock-chenille-bathrobe-u_img08_2026-05-27_195426.png | fw114thset_batch_04_small-heavy-dusty-rose-quadruple-peacock-chenille-bathrobe-u_img09_2026-05-27_195431.png</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>Screenshot 2026-05-27 at 7.53.49 PM.png: needs_review - Automatic crop passed layout checks. Possible Etsy overlay inside product photo. | Screenshot 2026-05-27 at 7.54.04 PM.png: needs_review - Crop width is outside expected product-photo range. | Screenshot 2026-05-27 at 7.54.10 PM.png: needs_review - Crop width is outside expected product-photo range.</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr"/>
-      <c r="M35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>fw115thset_batch_05</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Large lightweight "All American" vintage chenille bathrobe upcycled from'youth' hand tufted chenille bedspread Football moms/wives, this is your bathrobe! Looks like a football player kicking the</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Football moms/wives, this is your bathrobe! Looks like a football player kicking the
 football over the goal line. The bedspread is a 'youth' chenille, in the 1950s this was a
@@ -2890,59 +2819,59 @@
 wear over time that may take the form of thinning lines of chenille, skipped spots where</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>vintage, chenille, bathrobe, robe, upcycled, bedspread, cotton, hand tufted</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>large-lightweight-all-american-vintage-chenille-bathrobe-upcycled-from-youth-han</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>02_All_Listings_By_Set/fw115thset_batch_05/Cropped_Images</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>fw115thset_batch_05_large-lightweight-all-american-vintage-chenille-bathrobe-upc_img01_2026-05-27_195157.png</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>fw115thset_batch_05_large-lightweight-all-american-vintage-chenille-bathrobe-upc_img01_2026-05-27_195157.png | fw115thset_batch_05_large-lightweight-all-american-vintage-chenille-bathrobe-upc_img02_2026-05-27_195204.png | fw115thset_batch_05_large-lightweight-all-american-vintage-chenille-bathrobe-upc_img03_2026-05-27_195210.png | fw115thset_batch_05_large-lightweight-all-american-vintage-chenille-bathrobe-upc_img04_2026-05-27_195220.png | fw115thset_batch_05_large-lightweight-all-american-vintage-chenille-bathrobe-upc_img05_2026-05-27_195225.png | fw115thset_batch_05_large-lightweight-all-american-vintage-chenille-bathrobe-upc_img06_2026-05-27_195229.png | fw115thset_batch_05_large-lightweight-all-american-vintage-chenille-bathrobe-upc_img07_2026-05-27_195235.png | fw115thset_batch_05_large-lightweight-all-american-vintage-chenille-bathrobe-upc_img08_2026-05-27_195241.png | fw115thset_batch_05_large-lightweight-all-american-vintage-chenille-bathrobe-upc_img09_2026-05-27_195246.png</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>Screenshot 2026-05-27 at 7.51.57 PM.png: needs_review - Automatic crop passed layout checks. Possible Etsy overlay inside product photo.</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr"/>
-      <c r="M36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>fw116thset_batch_06</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Medium plush and heavy "Dawn in the Forest" peacock chenille bathrobe Upcycled from vintage hand tufted vintage chenille bedspreads</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Heavy chenille, plush tufting! Check out the tail, you cannot even see the3 backing
 under the tail it is so plush. Pretty colors, that forest green in the tail of the peacock
@@ -2960,55 +2889,55 @@
 chenille has come out; small pinholes, or variations in color. If any of these</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>vintage, chenille, bathrobe, robe, upcycled, bedspread, peacock, cotton, hand tufted, plush, heavy</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-bathrobe-upcycled-fro</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>02_All_Listings_By_Set/fw116thset_batch_06/Cropped_Images</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>fw116thset_batch_06_medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-b_img01_2026-05-27_200629.png</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>fw116thset_batch_06_medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-b_img01_2026-05-27_200629.png | fw116thset_batch_06_medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-b_img02_2026-05-27_200634.png | fw116thset_batch_06_medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-b_img03_2026-05-27_200639.png | fw116thset_batch_06_medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-b_img04_2026-05-27_200643.png | fw116thset_batch_06_medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-b_img05_2026-05-27_200723.png | fw116thset_batch_06_medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-b_img06_2026-05-27_200730.png | fw116thset_batch_06_medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-b_img07_2026-05-27_200742.png | fw116thset_batch_06_medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-b_img08_2026-05-27_200751.png | fw116thset_batch_06_medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-b_img09_2026-05-27_200804.png | fw116thset_batch_06_medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-b_img10_2026-05-27_200815.png | fw116thset_batch_06_medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-b_img11_2026-05-27_200823.png | fw116thset_batch_06_medium-plush-and-heavy-dawn-in-the-forest-peacock-chenille-b_img12_2026-05-27_200829.png</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr"/>
-      <c r="M37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>fw117thset_batch_07</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Medium plush and soft "Daisies at Sunset" vintage chenille bathrobe upcycled from rare purple hand tufted chenille bedspreads</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>The chenille this bathrobe was created from is soft and plush; in excellent vintage shape.
 Purple on purple, very rare; not many of this color combo in my shop or in existance,
@@ -3026,59 +2955,59 @@
 The nraduntion of chenille conned in the Ilnited Statec after ahnut 10kN and much of it</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>vintage, chenille, bathrobe, robe, upcycled, bedspread, cotton, hand tufted, plush</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>medium-plush-and-soft-daisies-at-sunset-vintage-chenille-bathrobe-upcycled-from</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>02_All_Listings_By_Set/fw117thset_batch_07/Cropped_Images</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>fw117thset_batch_07_medium-plush-and-soft-daisies-at-sunset-vintage-chenille-bat_img01_2026-05-28_074639.png</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>fw117thset_batch_07_medium-plush-and-soft-daisies-at-sunset-vintage-chenille-bat_img01_2026-05-28_074639.png | fw117thset_batch_07_medium-plush-and-soft-daisies-at-sunset-vintage-chenille-bat_img02_2026-05-28_074644.png | fw117thset_batch_07_medium-plush-and-soft-daisies-at-sunset-vintage-chenille-bat_img03_2026-05-28_074649.png | fw117thset_batch_07_medium-plush-and-soft-daisies-at-sunset-vintage-chenille-bat_img04_2026-05-28_074654.png | fw117thset_batch_07_medium-plush-and-soft-daisies-at-sunset-vintage-chenille-bat_img05_2026-05-28_074659.png | fw117thset_batch_07_medium-plush-and-soft-daisies-at-sunset-vintage-chenille-bat_img06_2026-05-28_074703.png | fw117thset_batch_07_medium-plush-and-soft-daisies-at-sunset-vintage-chenille-bat_img07_2026-05-28_074708.png | fw117thset_batch_07_medium-plush-and-soft-daisies-at-sunset-vintage-chenille-bat_img08_2026-05-28_074713.png</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>Screenshot 2026-05-28 at 7.46.39 AM.png: needs_review - Automatic crop passed layout checks. Possible Etsy overlay inside product photo.</t>
         </is>
       </c>
-      <c r="L38" s="2" t="inlineStr"/>
-      <c r="M38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>fw119thset_batch_08</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Large Uber plush and heavy "Midnight Blooms" chenille bathrobe upcycled from vintage hand tufted chenille bedspreads Thio roudl hluo id poro in chanilla, doronidlya0₺hathad eotniu0d$t0 ünh ddd aur timo!</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>This royal blue is rare in chenille; especially one that has retained its rich color over time!
 The chenille in this robe is so plush, I broke 3 machine needles sewing it! Absolutely
@@ -3095,29 +3024,86 @@
 finite, it has become more difficult to find! Although chenille is durable, it can suffer</t>
         </is>
       </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>vintage, chenille, bathrobe, robe, upcycled, bedspread, flower, cotton, hand tufted, plush, heavy</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe-upcycled-from-vinta</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>02_All_Listings_By_Set/fw119thset_batch_08/Cropped_Images</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img01_2026-05-28_074436.png</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img01_2026-05-28_074436.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img02_2026-05-28_074441.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img03_2026-05-28_074445.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img04_2026-05-28_074450.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img05_2026-05-28_074454.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img06_2026-05-28_074458.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img07_2026-05-28_074503.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img08_2026-05-28_074508.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img09_2026-05-28_074512.png</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Screenshot 2026-05-28 at 7.44.36 AM.png: needs_review - Automatic crop passed layout checks. Possible Etsy overlay inside product photo.</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>fw120thset_batch_01</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Large heavy “Border Flowers” vintage chenille bathrobe upcycled from combo hobnail and chenille bedspread</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>More later</t>
+        </is>
+      </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>vintage, chenille, bathrobe, robe, upcycled, bedspread, flower, cotton, hand tufted, plush, heavy</t>
+          <t>vintage, chenille, bathrobe, robe, upcycled, bedspread, hobnail, flower, heavy</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe-upcycled-from-vinta</t>
+          <t>large-heavy-border-flowers-vintage-chenille-bathrobe-upcycled-from-combo-hobnail</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>02_All_Listings_By_Set/fw119thset_batch_08/Cropped_Images</t>
+          <t>02_All_Listings_By_Set/fw120thset_batch_01/Cropped_Images</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img01_2026-05-28_074436.png</t>
+          <t>fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img01_2026-05-28_075529.png</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img01_2026-05-28_074436.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img02_2026-05-28_074441.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img03_2026-05-28_074445.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img04_2026-05-28_074450.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img05_2026-05-28_074454.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img06_2026-05-28_074458.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img07_2026-05-28_074503.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img08_2026-05-28_074508.png | fw119thset_batch_08_large-uber-plush-and-heavy-midnight-blooms-chenille-bathrobe_img09_2026-05-28_074512.png</t>
+          <t>fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img01_2026-05-28_075529.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img02_2026-05-28_075534.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img03_2026-05-28_075539.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img04_2026-05-28_075544.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img05_2026-05-28_075549.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img06_2026-05-28_075553.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img07_2026-05-28_075558.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img08_2026-05-28_075603.png</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3127,7 +3113,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Screenshot 2026-05-28 at 7.44.36 AM.png: needs_review - Automatic crop passed layout checks. Possible Etsy overlay inside product photo.</t>
+          <t>Screenshot 2026-05-28 at 7.55.29 AM.png: needs_review - Automatic crop passed layout checks. Possible Etsy overlay inside product photo.</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr"/>
@@ -3139,12 +3125,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>fw120thset_batch_01</t>
+          <t>fw121stset_batch_09</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Large heavy “Border Flowers” vintage chenille bathrobe upcycled from combo hobnail and chenille bedspread</t>
+          <t>Large heavy "Border Flowers" vintage chenille bathrobe upcycled from combo hobnail and chenille bedspread</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -3164,17 +3150,17 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>02_All_Listings_By_Set/fw120thset_batch_01/Cropped_Images</t>
+          <t>02_All_Listings_By_Set/fw121stset_batch_09/Cropped_Images</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img01_2026-05-28_075529.png</t>
+          <t>fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img01_2026-05-28_075422.png</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img01_2026-05-28_075529.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img02_2026-05-28_075534.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img03_2026-05-28_075539.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img04_2026-05-28_075544.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img05_2026-05-28_075549.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img06_2026-05-28_075553.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img07_2026-05-28_075558.png | fw120thset_batch_01_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img08_2026-05-28_075603.png</t>
+          <t>fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img01_2026-05-28_075422.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img02_2026-05-28_075427.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img03_2026-05-28_075432.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img04_2026-05-28_075436.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img05_2026-05-28_075440.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img06_2026-05-28_075444.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img07_2026-05-28_075449.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img08_2026-05-28_075453.png</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -3184,7 +3170,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Screenshot 2026-05-28 at 7.55.29 AM.png: needs_review - Automatic crop passed layout checks. Possible Etsy overlay inside product photo.</t>
+          <t>Screenshot 2026-05-28 at 7.54.22 AM.png: needs_review - Automatic crop passed layout checks. Possible Etsy overlay inside product photo.</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr"/>
@@ -3196,72 +3182,15 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>fw121stset_batch_09</t>
+          <t>fw122ndset_batch_10</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Large heavy "Border Flowers" vintage chenille bathrobe upcycled from combo hobnail and chenille bedspread</t>
+          <t>L midlength soft "Sassy Fringed" vintage chenille bathrobe upcycled from handtufted hobnail and regular hand tufted chenille bedspreads</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>More later</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>vintage, chenille, bathrobe, robe, upcycled, bedspread, hobnail, flower, heavy</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>large-heavy-border-flowers-vintage-chenille-bathrobe-upcycled-from-combo-hobnail</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>02_All_Listings_By_Set/fw121stset_batch_09/Cropped_Images</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img01_2026-05-28_075422.png</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img01_2026-05-28_075422.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img02_2026-05-28_075427.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img03_2026-05-28_075432.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img04_2026-05-28_075436.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img05_2026-05-28_075440.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img06_2026-05-28_075444.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img07_2026-05-28_075449.png | fw121stset_batch_09_large-heavy-border-flowers-vintage-chenille-bathrobe-upcycle_img08_2026-05-28_075453.png</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>Screenshot 2026-05-28 at 7.54.22 AM.png: needs_review - Automatic crop passed layout checks. Possible Etsy overlay inside product photo.</t>
-        </is>
-      </c>
-      <c r="L41" s="2" t="inlineStr"/>
-      <c r="M41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>fw122ndset_batch_10</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>L midlength soft "Sassy Fringed" vintage chenille bathrobe upcycled from handtufted hobnail and regular hand tufted chenille bedspreads</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>The vintage chenille I used to create this unusual bathrobe is a classic design, I cut it a
 bit shorter (should fall just below the knees) so that I could capture and incorporate
@@ -3280,43 +3209,43 @@
 11)</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>vintage, chenille, bathrobe, robe, upcycled, bedspread, hobnail, cotton, hand tufted</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>l-midlength-soft-sassy-fringed-vintage-chenille-bathrobe-upcycled-from-handtufte</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>02_All_Listings_By_Set/fw122ndset_batch_10/Cropped_Images</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>fw122ndset_batch_10_l-midlength-soft-sassy-fringed-vintage-chenille-bathrobe-upc_img01_2026-05-28_075252.png</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>fw122ndset_batch_10_l-midlength-soft-sassy-fringed-vintage-chenille-bathrobe-upc_img01_2026-05-28_075252.png | fw122ndset_batch_10_l-midlength-soft-sassy-fringed-vintage-chenille-bathrobe-upc_img02_2026-05-28_075300.png | fw122ndset_batch_10_l-midlength-soft-sassy-fringed-vintage-chenille-bathrobe-upc_img03_2026-05-28_075305.png | fw122ndset_batch_10_l-midlength-soft-sassy-fringed-vintage-chenille-bathrobe-upc_img04_2026-05-28_075309.png | fw122ndset_batch_10_l-midlength-soft-sassy-fringed-vintage-chenille-bathrobe-upc_img05_2026-05-28_075313.png | fw122ndset_batch_10_l-midlength-soft-sassy-fringed-vintage-chenille-bathrobe-upc_img06_2026-05-28_075320.png | fw122ndset_batch_10_l-midlength-soft-sassy-fringed-vintage-chenille-bathrobe-upc_img07_2026-05-28_075325.png | fw122ndset_batch_10_l-midlength-soft-sassy-fringed-vintage-chenille-bathrobe-upc_img08_2026-05-28_075330.png | fw122ndset_batch_10_l-midlength-soft-sassy-fringed-vintage-chenille-bathrobe-upc_img09_2026-05-28_075335.png</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>Screenshot 2026-05-28 at 7.52.52 AM.png: needs_review - Automatic crop passed layout checks. Possible Etsy overlay inside product photo. | Screenshot 2026-05-28 at 7.53.20 AM.png: needs_review - Crop width is outside expected product-photo range.</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr"/>
-      <c r="M42" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M42"/>

</xml_diff>